<commit_message>
Add Batch 2 Sony H1 tags; update Batch 1 with newly identified parts
Claude-Session: https://claude.ai/code/session_01GqspcdoB39p9nTcqgMudzj
</commit_message>
<xml_diff>
--- a/Batch_1_H1_tags.xlsx
+++ b/Batch_1_H1_tags.xlsx
@@ -3785,15 +3785,19 @@
           <t xml:space="preserve">Sony </t>
         </is>
       </c>
-      <c r="C77" s="2" t="inlineStr"/>
-      <c r="D77" s="9" t="inlineStr">
-        <is>
-          <t>Not searched</t>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Sony TV Stand Base Right - 5-023-428-01</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E77" s="2" t="inlineStr">
         <is>
-          <t>Search limit reached before this part was looked up</t>
+          <t>Paired with 5-023-427-01 for XR-65A80J</t>
         </is>
       </c>
       <c r="F77" s="2" t="n"/>
@@ -3829,15 +3833,19 @@
           <t xml:space="preserve">Sony </t>
         </is>
       </c>
-      <c r="C78" s="2" t="inlineStr"/>
-      <c r="D78" s="9" t="inlineStr">
-        <is>
-          <t>Not searched</t>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Sony Panel B Assembly - A-2203-126-B</t>
+        </is>
+      </c>
+      <c r="D78" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Search limit reached before this part was looked up</t>
+          <t>Single listing; device not stated</t>
         </is>
       </c>
       <c r="F78" s="2" t="n"/>
@@ -4093,17 +4101,17 @@
           <t xml:space="preserve">Sony </t>
         </is>
       </c>
-      <c r="C84" s="2" t="inlineStr"/>
-      <c r="D84" s="9" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E84" s="2" t="inlineStr">
-        <is>
-          <t>Search limit reached before this part was looked up</t>
-        </is>
-      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Sony Headphone Carrying Case (WH-1000XM5) - 5-036-014-01</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr"/>
       <c r="F84" s="2" t="n"/>
       <c r="G84" s="2" t="n"/>
       <c r="H84" s="2" t="n"/>
@@ -4313,17 +4321,17 @@
           <t xml:space="preserve">Sony </t>
         </is>
       </c>
-      <c r="C89" s="2" t="inlineStr"/>
-      <c r="D89" s="9" t="inlineStr">
-        <is>
-          <t>Not searched</t>
-        </is>
-      </c>
-      <c r="E89" s="2" t="inlineStr">
-        <is>
-          <t>Search limit reached before this part was looked up</t>
-        </is>
-      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Sony TV Main Board BMFW - A-2072-545-C</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr"/>
       <c r="F89" s="2" t="n"/>
       <c r="G89" s="2" t="n"/>
       <c r="H89" s="2" t="n"/>

</xml_diff>